<commit_message>
Cập nhật exe để không cần cài python ở máy khách hàng
</commit_message>
<xml_diff>
--- a/IIS/ExcelCauHinh/Settup AXE.xlsx
+++ b/IIS/ExcelCauHinh/Settup AXE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\ToolAXE\CauHinhHeThongAXE\IIS\ExcelCauHinh\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B33C765-5D55-4437-8890-99157C97562F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{600775A8-B483-43AF-87EF-8D6F340B82FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cài đặt IIS" sheetId="2" r:id="rId1"/>
@@ -336,13 +336,13 @@
     <t>AXE_Test_</t>
   </si>
   <si>
-    <t>E:\SourceCodeAXE\</t>
-  </si>
-  <si>
     <t>C:\Users\Admin\Desktop\Test</t>
   </si>
   <si>
     <t>http://localhost:1221</t>
+  </si>
+  <si>
+    <t>E:\TestTool_Dựng web\</t>
   </si>
 </sst>
 </file>
@@ -631,50 +631,50 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -988,15 +988,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
       <c r="G1" s="12"/>
-      <c r="H1" s="45"/>
-      <c r="I1" s="45"/>
-      <c r="J1" s="45"/>
+      <c r="H1" s="39"/>
+      <c r="I1" s="39"/>
+      <c r="J1" s="39"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
@@ -1009,7 +1009,7 @@
         <v>3</v>
       </c>
       <c r="G2" s="12"/>
-      <c r="H2" s="46"/>
+      <c r="H2" s="40"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
@@ -1020,20 +1020,20 @@
       </c>
       <c r="C3" s="17"/>
       <c r="G3" s="12"/>
-      <c r="H3" s="47"/>
+      <c r="H3" s="41"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="15" t="s">
         <v>5</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C4" s="17" t="s">
         <v>6</v>
       </c>
       <c r="G4" s="12"/>
-      <c r="H4" s="47"/>
+      <c r="H4" s="41"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="15" t="s">
@@ -1044,33 +1044,33 @@
       </c>
       <c r="C5" s="17"/>
       <c r="G5" s="12"/>
-      <c r="H5" s="47"/>
+      <c r="H5" s="41"/>
     </row>
     <row r="6" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A6" s="18" t="s">
         <v>8</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C6" s="17" t="s">
         <v>9</v>
       </c>
       <c r="G6" s="12"/>
-      <c r="H6" s="47"/>
+      <c r="H6" s="41"/>
     </row>
     <row r="7" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A7" s="18" t="s">
         <v>10</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C7" s="17" t="s">
         <v>9</v>
       </c>
       <c r="G7" s="12"/>
-      <c r="H7" s="47"/>
+      <c r="H7" s="41"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="18" t="s">
@@ -1081,17 +1081,17 @@
       </c>
       <c r="C8" s="17"/>
       <c r="G8" s="12"/>
-      <c r="H8" s="48"/>
+      <c r="H8" s="42"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="37" t="s">
+      <c r="A9" s="47" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="38"/>
-      <c r="C9" s="38"/>
-      <c r="D9" s="38"/>
-      <c r="E9" s="38"/>
-      <c r="F9" s="38"/>
+      <c r="B9" s="48"/>
+      <c r="C9" s="48"/>
+      <c r="D9" s="48"/>
+      <c r="E9" s="48"/>
+      <c r="F9" s="48"/>
       <c r="G9" s="12"/>
       <c r="H9" s="20"/>
     </row>
@@ -1133,14 +1133,14 @@
       <c r="H12" s="21"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="45" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="40"/>
-      <c r="C13" s="40"/>
-      <c r="D13" s="40"/>
-      <c r="E13" s="40"/>
-      <c r="F13" s="41"/>
+      <c r="B13" s="46"/>
+      <c r="C13" s="46"/>
+      <c r="D13" s="46"/>
+      <c r="E13" s="46"/>
+      <c r="F13" s="50"/>
       <c r="G13" s="12"/>
       <c r="H13" s="13"/>
     </row>
@@ -1173,7 +1173,7 @@
       </c>
       <c r="B15" s="21" t="str">
         <f>$B$4&amp;"AXE-Dash"</f>
-        <v>E:\SourceCodeAXE\AXE-Dash</v>
+        <v>E:\TestTool_Dựng web\AXE-Dash</v>
       </c>
       <c r="C15" s="17" t="s">
         <v>25</v>
@@ -1189,7 +1189,7 @@
       <c r="G15" s="12"/>
       <c r="H15" s="21" t="str">
         <f>IF(A15="","",$B$8&amp;" add site /name:"""&amp;A15&amp;""" /physicalPath:"&amp;B15&amp;" /bindings:"&amp;C15&amp;"/*:"&amp;D15&amp;":"&amp;E15&amp;"" )</f>
-        <v>c:\Windows\system32\inetsrv\appcmd add site /name:"AXE_Test_Web" /physicalPath:E:\SourceCodeAXE\AXE-Dash /bindings:http/*:1221:</v>
+        <v>c:\Windows\system32\inetsrv\appcmd add site /name:"AXE_Test_Web" /physicalPath:E:\TestTool_Dựng web\AXE-Dash /bindings:http/*:1221:</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
@@ -1203,14 +1203,14 @@
       <c r="H16" s="21"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="45" t="s">
         <v>26</v>
       </c>
-      <c r="B17" s="40"/>
-      <c r="C17" s="40"/>
-      <c r="D17" s="40"/>
-      <c r="E17" s="40"/>
-      <c r="F17" s="40"/>
+      <c r="B17" s="46"/>
+      <c r="C17" s="46"/>
+      <c r="D17" s="46"/>
+      <c r="E17" s="46"/>
+      <c r="F17" s="46"/>
       <c r="G17" s="12"/>
       <c r="H17" s="13"/>
     </row>
@@ -1244,19 +1244,19 @@
       </c>
       <c r="C19" s="17" t="str">
         <f>$B$4&amp;"AXE-Acc"</f>
-        <v>E:\SourceCodeAXE\AXE-Acc</v>
+        <v>E:\TestTool_Dựng web\AXE-Acc</v>
       </c>
       <c r="D19" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="E19" s="36" t="s">
+      <c r="E19" s="49" t="s">
         <v>33</v>
       </c>
-      <c r="F19" s="36"/>
+      <c r="F19" s="49"/>
       <c r="G19" s="12"/>
       <c r="H19" s="21" t="str">
         <f t="shared" ref="H19:H24" si="1">IF(D19="","",$B$8&amp;" add app  /site.name:"""&amp;B19&amp;""" /path:/"&amp;A19&amp;" /physicalPath:"&amp;C19&amp;"")</f>
-        <v>c:\Windows\system32\inetsrv\appcmd add app  /site.name:"AXE_Test_Web" /path:/login /physicalPath:E:\SourceCodeAXE\AXE-Acc</v>
+        <v>c:\Windows\system32\inetsrv\appcmd add app  /site.name:"AXE_Test_Web" /path:/login /physicalPath:E:\TestTool_Dựng web\AXE-Acc</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="27.6" x14ac:dyDescent="0.25">
@@ -1269,19 +1269,19 @@
       </c>
       <c r="C20" s="17" t="str">
         <f>$B$4&amp;"AXE-Admin"</f>
-        <v>E:\SourceCodeAXE\AXE-Admin</v>
+        <v>E:\TestTool_Dựng web\AXE-Admin</v>
       </c>
       <c r="D20" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="E20" s="36" t="s">
+      <c r="E20" s="49" t="s">
         <v>33</v>
       </c>
-      <c r="F20" s="36"/>
+      <c r="F20" s="49"/>
       <c r="G20" s="12"/>
       <c r="H20" s="21" t="str">
         <f t="shared" si="1"/>
-        <v>c:\Windows\system32\inetsrv\appcmd add app  /site.name:"AXE_Test_Web" /path:/admin /physicalPath:E:\SourceCodeAXE\AXE-Admin</v>
+        <v>c:\Windows\system32\inetsrv\appcmd add app  /site.name:"AXE_Test_Web" /path:/admin /physicalPath:E:\TestTool_Dựng web\AXE-Admin</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="27.6" x14ac:dyDescent="0.25">
@@ -1294,19 +1294,19 @@
       </c>
       <c r="C21" s="17" t="str">
         <f>$B$4&amp;"AXE-ResumUploader"</f>
-        <v>E:\SourceCodeAXE\AXE-ResumUploader</v>
+        <v>E:\TestTool_Dựng web\AXE-ResumUploader</v>
       </c>
       <c r="D21" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="E21" s="36" t="s">
+      <c r="E21" s="49" t="s">
         <v>33</v>
       </c>
-      <c r="F21" s="36"/>
+      <c r="F21" s="49"/>
       <c r="G21" s="12"/>
       <c r="H21" s="21" t="str">
         <f t="shared" si="1"/>
-        <v>c:\Windows\system32\inetsrv\appcmd add app  /site.name:"AXE_Test_Web" /path:/resumable /physicalPath:E:\SourceCodeAXE\AXE-ResumUploader</v>
+        <v>c:\Windows\system32\inetsrv\appcmd add app  /site.name:"AXE_Test_Web" /path:/resumable /physicalPath:E:\TestTool_Dựng web\AXE-ResumUploader</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="27.6" x14ac:dyDescent="0.25">
@@ -1319,19 +1319,19 @@
       </c>
       <c r="C22" s="17" t="str">
         <f>$B$4&amp;"AXE-Uploader"</f>
-        <v>E:\SourceCodeAXE\AXE-Uploader</v>
+        <v>E:\TestTool_Dựng web\AXE-Uploader</v>
       </c>
       <c r="D22" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="E22" s="36" t="s">
+      <c r="E22" s="49" t="s">
         <v>33</v>
       </c>
-      <c r="F22" s="36"/>
+      <c r="F22" s="49"/>
       <c r="G22" s="12"/>
       <c r="H22" s="21" t="str">
         <f t="shared" si="1"/>
-        <v>c:\Windows\system32\inetsrv\appcmd add app  /site.name:"AXE_Test_Web" /path:/uploader /physicalPath:E:\SourceCodeAXE\AXE-Uploader</v>
+        <v>c:\Windows\system32\inetsrv\appcmd add app  /site.name:"AXE_Test_Web" /path:/uploader /physicalPath:E:\TestTool_Dựng web\AXE-Uploader</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
@@ -1349,10 +1349,10 @@
       <c r="D23" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="E23" s="36" t="s">
+      <c r="E23" s="49" t="s">
         <v>33</v>
       </c>
-      <c r="F23" s="36"/>
+      <c r="F23" s="49"/>
       <c r="G23" s="12"/>
       <c r="H23" s="21" t="str">
         <f t="shared" si="1"/>
@@ -1369,19 +1369,19 @@
       </c>
       <c r="C24" s="17" t="str">
         <f>$B$4&amp;"AXE-SoHoa"</f>
-        <v>E:\SourceCodeAXE\AXE-SoHoa</v>
+        <v>E:\TestTool_Dựng web\AXE-SoHoa</v>
       </c>
       <c r="D24" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="E24" s="36" t="s">
+      <c r="E24" s="49" t="s">
         <v>39</v>
       </c>
-      <c r="F24" s="36"/>
+      <c r="F24" s="49"/>
       <c r="G24" s="12"/>
       <c r="H24" s="21" t="str">
         <f t="shared" si="1"/>
-        <v>c:\Windows\system32\inetsrv\appcmd add app  /site.name:"AXE_Test_Web" /path:/doc /physicalPath:E:\SourceCodeAXE\AXE-SoHoa</v>
+        <v>c:\Windows\system32\inetsrv\appcmd add app  /site.name:"AXE_Test_Web" /path:/doc /physicalPath:E:\TestTool_Dựng web\AXE-SoHoa</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
@@ -1389,20 +1389,20 @@
       <c r="B25" s="21"/>
       <c r="C25" s="17"/>
       <c r="D25" s="21"/>
-      <c r="E25" s="36"/>
-      <c r="F25" s="36"/>
+      <c r="E25" s="49"/>
+      <c r="F25" s="49"/>
       <c r="G25" s="12"/>
       <c r="H25" s="21"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="37" t="s">
+      <c r="A26" s="47" t="s">
         <v>40</v>
       </c>
-      <c r="B26" s="38"/>
-      <c r="C26" s="38"/>
-      <c r="D26" s="38"/>
-      <c r="E26" s="38"/>
-      <c r="F26" s="38"/>
+      <c r="B26" s="48"/>
+      <c r="C26" s="48"/>
+      <c r="D26" s="48"/>
+      <c r="E26" s="48"/>
+      <c r="F26" s="48"/>
       <c r="H26" s="13"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
@@ -1439,14 +1439,14 @@
       <c r="H29" s="21"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="45" t="s">
+      <c r="A30" s="39" t="s">
         <v>42</v>
       </c>
-      <c r="B30" s="45"/>
-      <c r="C30" s="45"/>
-      <c r="D30" s="45"/>
-      <c r="E30" s="45"/>
-      <c r="F30" s="45"/>
+      <c r="B30" s="39"/>
+      <c r="C30" s="39"/>
+      <c r="D30" s="39"/>
+      <c r="E30" s="39"/>
+      <c r="F30" s="39"/>
       <c r="H30" s="21"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
@@ -1459,11 +1459,11 @@
       <c r="C31" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="D31" s="50" t="s">
+      <c r="D31" s="44" t="s">
         <v>3</v>
       </c>
-      <c r="E31" s="50"/>
-      <c r="F31" s="50"/>
+      <c r="E31" s="44"/>
+      <c r="F31" s="44"/>
       <c r="H31" s="21"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
@@ -1478,9 +1478,9 @@
         <f>$A$11</f>
         <v>AXE_Test-Web</v>
       </c>
-      <c r="D32" s="36"/>
-      <c r="E32" s="36"/>
-      <c r="F32" s="36"/>
+      <c r="D32" s="49"/>
+      <c r="E32" s="49"/>
+      <c r="F32" s="49"/>
       <c r="H32" s="21" t="str">
         <f>IF(C32="","",$B$8&amp;" set app "&amp;A32&amp;"/"&amp;B32&amp;"  /"&amp;"applicationPool:"&amp;C32&amp;"")</f>
         <v>c:\Windows\system32\inetsrv\appcmd set app AXE_Test_Web/login  /applicationPool:AXE_Test-Web</v>
@@ -1498,9 +1498,9 @@
         <f t="shared" ref="C33:C37" si="3">$A$11</f>
         <v>AXE_Test-Web</v>
       </c>
-      <c r="D33" s="49"/>
-      <c r="E33" s="49"/>
-      <c r="F33" s="49"/>
+      <c r="D33" s="43"/>
+      <c r="E33" s="43"/>
+      <c r="F33" s="43"/>
       <c r="H33" s="21" t="str">
         <f>IF(C33="","",$B$8&amp;" set app "&amp;A33&amp;"/"&amp;B33&amp;"  /"&amp;"applicationPool:"&amp;C33&amp;"")</f>
         <v>c:\Windows\system32\inetsrv\appcmd set app AXE_Test_Web/admin  /applicationPool:AXE_Test-Web</v>
@@ -1518,9 +1518,9 @@
         <f t="shared" si="3"/>
         <v>AXE_Test-Web</v>
       </c>
-      <c r="D34" s="49"/>
-      <c r="E34" s="49"/>
-      <c r="F34" s="49"/>
+      <c r="D34" s="43"/>
+      <c r="E34" s="43"/>
+      <c r="F34" s="43"/>
       <c r="H34" s="21" t="str">
         <f>IF(C34="","",$B$8&amp;" set app "&amp;A34&amp;"/"&amp;B34&amp;"  /"&amp;"applicationPool:"&amp;C34&amp;"")</f>
         <v>c:\Windows\system32\inetsrv\appcmd set app AXE_Test_Web/resumable  /applicationPool:AXE_Test-Web</v>
@@ -1538,9 +1538,9 @@
         <f t="shared" si="3"/>
         <v>AXE_Test-Web</v>
       </c>
-      <c r="D35" s="49"/>
-      <c r="E35" s="49"/>
-      <c r="F35" s="49"/>
+      <c r="D35" s="43"/>
+      <c r="E35" s="43"/>
+      <c r="F35" s="43"/>
       <c r="H35" s="21" t="str">
         <f>IF(C35="","",$B$8&amp;" set app "&amp;A35&amp;"/"&amp;B35&amp;"  /"&amp;"applicationPool:"&amp;C35&amp;"")</f>
         <v>c:\Windows\system32\inetsrv\appcmd set app AXE_Test_Web/uploader  /applicationPool:AXE_Test-Web</v>
@@ -1558,9 +1558,9 @@
         <f t="shared" si="3"/>
         <v>AXE_Test-Web</v>
       </c>
-      <c r="D36" s="49"/>
-      <c r="E36" s="49"/>
-      <c r="F36" s="49"/>
+      <c r="D36" s="43"/>
+      <c r="E36" s="43"/>
+      <c r="F36" s="43"/>
       <c r="H36" s="21" t="str">
         <f>IF(C36="","","c:\Windows\system32\inetsrv\appcmd set app "&amp;A36&amp;"/"&amp;B36&amp;"  /"&amp;"applicationPool:"&amp;C36&amp;"")</f>
         <v>c:\Windows\system32\inetsrv\appcmd set app AXE_Test_Web/storage  /applicationPool:AXE_Test-Web</v>
@@ -1578,9 +1578,9 @@
         <f t="shared" si="3"/>
         <v>AXE_Test-Web</v>
       </c>
-      <c r="D37" s="42"/>
-      <c r="E37" s="43"/>
-      <c r="F37" s="44"/>
+      <c r="D37" s="36"/>
+      <c r="E37" s="37"/>
+      <c r="F37" s="38"/>
       <c r="H37" s="21" t="str">
         <f t="shared" ref="H37:H38" si="4">IF(C37="","","c:\Windows\system32\inetsrv\appcmd set app "&amp;A37&amp;"/"&amp;B37&amp;"  /"&amp;"applicationPool:"&amp;C37&amp;"")</f>
         <v>c:\Windows\system32\inetsrv\appcmd set app AXE_Test_Web/doc  /applicationPool:AXE_Test-Web</v>
@@ -1590,9 +1590,9 @@
       <c r="A38" s="21"/>
       <c r="B38" s="21"/>
       <c r="C38" s="17"/>
-      <c r="D38" s="42"/>
-      <c r="E38" s="43"/>
-      <c r="F38" s="44"/>
+      <c r="D38" s="36"/>
+      <c r="E38" s="37"/>
+      <c r="F38" s="38"/>
       <c r="H38" s="21" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -1600,6 +1600,13 @@
     </row>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="A9:F9"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="E23:F23"/>
     <mergeCell ref="D37:F37"/>
     <mergeCell ref="D38:F38"/>
     <mergeCell ref="H1:J1"/>
@@ -1616,13 +1623,6 @@
     <mergeCell ref="D35:F35"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="E19:F19"/>
-    <mergeCell ref="E25:F25"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="A9:F9"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="E23:F23"/>
   </mergeCells>
   <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K427:K1048576 G26:G426 K1:K25 B18 G9:G10" xr:uid="{00000000-0002-0000-0000-000000000000}">
@@ -1666,11 +1666,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
       <c r="D1" s="26"/>
       <c r="E1" s="26"/>
       <c r="F1" s="12"/>
@@ -1689,7 +1689,7 @@
       <c r="D2" s="31"/>
       <c r="E2" s="31"/>
       <c r="F2" s="12"/>
-      <c r="G2" s="46"/>
+      <c r="G2" s="40"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
@@ -1700,7 +1700,7 @@
       </c>
       <c r="C3" s="21"/>
       <c r="F3" s="12"/>
-      <c r="G3" s="47"/>
+      <c r="G3" s="41"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="15" t="s">
@@ -1711,7 +1711,7 @@
       </c>
       <c r="C4" s="21"/>
       <c r="F4" s="12"/>
-      <c r="G4" s="47"/>
+      <c r="G4" s="41"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="15" t="s">
@@ -1722,7 +1722,7 @@
       </c>
       <c r="C5" s="21"/>
       <c r="F5" s="12"/>
-      <c r="G5" s="47"/>
+      <c r="G5" s="41"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="18" t="s">
@@ -1733,14 +1733,14 @@
       </c>
       <c r="C6" s="21"/>
       <c r="F6" s="12"/>
-      <c r="G6" s="47"/>
+      <c r="G6" s="41"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="37" t="s">
+      <c r="A7" s="47" t="s">
         <v>51</v>
       </c>
-      <c r="B7" s="38"/>
-      <c r="C7" s="38"/>
+      <c r="B7" s="48"/>
+      <c r="C7" s="48"/>
       <c r="D7" s="26"/>
       <c r="E7" s="26"/>
       <c r="F7" s="12"/>
@@ -1774,11 +1774,11 @@
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="37" t="s">
+      <c r="A10" s="47" t="s">
         <v>53</v>
       </c>
-      <c r="B10" s="38"/>
-      <c r="C10" s="38"/>
+      <c r="B10" s="48"/>
+      <c r="C10" s="48"/>
       <c r="D10" s="26"/>
       <c r="E10" s="26"/>
       <c r="F10" s="12"/>
@@ -1804,11 +1804,11 @@
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="45" t="s">
         <v>55</v>
       </c>
-      <c r="B13" s="40"/>
-      <c r="C13" s="40"/>
+      <c r="B13" s="46"/>
+      <c r="C13" s="46"/>
       <c r="D13" s="26"/>
       <c r="E13" s="26"/>
       <c r="F13" s="12"/>
@@ -2831,6 +2831,27 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Ghich_x00fa_ xmlns="97d068c0-5bfb-413b-9996-819e39fdf128" xsi:nil="true"/>
+    <TaxCatchAll xmlns="2c7f0914-2907-4374-a90b-da4fc7d9e6d0" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="97d068c0-5bfb-413b-9996-819e39fdf128">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010097FE9C0C8E574444875F1CBBF8414DDA" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c7e0992f45b677c2156c5ab52d17057f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="97d068c0-5bfb-413b-9996-819e39fdf128" xmlns:ns3="2c7f0914-2907-4374-a90b-da4fc7d9e6d0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2f06a3ea3329379ac3c4a4f5da7fed49" ns2:_="" ns3:_="">
     <xsd:import namespace="97d068c0-5bfb-413b-9996-819e39fdf128"/>
@@ -3065,28 +3086,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Ghich_x00fa_ xmlns="97d068c0-5bfb-413b-9996-819e39fdf128" xsi:nil="true"/>
-    <TaxCatchAll xmlns="2c7f0914-2907-4374-a90b-da4fc7d9e6d0" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="97d068c0-5bfb-413b-9996-819e39fdf128">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1FDEE16B-9D1D-4FD0-B127-E14D995BDF2D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EA8505A6-C0ED-439D-B023-AA9B1B1662BB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="97d068c0-5bfb-413b-9996-819e39fdf128"/>
+    <ds:schemaRef ds:uri="2c7f0914-2907-4374-a90b-da4fc7d9e6d0"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E3A15DF-6B1B-40AC-992D-CB264AF46DCF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3103,23 +3122,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EA8505A6-C0ED-439D-B023-AA9B1B1662BB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="97d068c0-5bfb-413b-9996-819e39fdf128"/>
-    <ds:schemaRef ds:uri="2c7f0914-2907-4374-a90b-da4fc7d9e6d0"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1FDEE16B-9D1D-4FD0-B127-E14D995BDF2D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Cập nhật setup môi trường iis và sql server
</commit_message>
<xml_diff>
--- a/IIS/ExcelCauHinh/Settup AXE.xlsx
+++ b/IIS/ExcelCauHinh/Settup AXE.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\ToolAXE\CauHinhHeThongAXE\IIS\ExcelCauHinh\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{600775A8-B483-43AF-87EF-8D6F340B82FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57508721-09F3-4CFC-8249-C1A03383E5A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -330,19 +330,19 @@
     <t>Tạo Application Pool cho Website/Application</t>
   </si>
   <si>
-    <t>AXE_Test</t>
-  </si>
-  <si>
-    <t>AXE_Test_</t>
-  </si>
-  <si>
-    <t>C:\Users\Admin\Desktop\Test</t>
-  </si>
-  <si>
-    <t>http://localhost:1221</t>
-  </si>
-  <si>
-    <t>E:\TestTool_Dựng web\</t>
+    <t>AXE_THAINGUYEN</t>
+  </si>
+  <si>
+    <t>AXE_2026_THAINGUYEN_</t>
+  </si>
+  <si>
+    <t>E:\Source_Web\AXE-2026-ThaiNguyen\</t>
+  </si>
+  <si>
+    <t>http://localhost:8539</t>
+  </si>
+  <si>
+    <t>E:\DataStorage\StorageAXE-2026-ThaiNguyen\Storage</t>
   </si>
 </sst>
 </file>
@@ -973,8 +973,8 @@
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34" style="11" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="49.44140625" style="11" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.109375" style="25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="57.88671875" style="11" customWidth="1"/>
+    <col min="3" max="3" width="46" style="25" customWidth="1"/>
     <col min="4" max="5" width="7.88671875" style="11" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="20.6640625" style="11" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="5.33203125" style="11" bestFit="1" customWidth="1"/>
@@ -1027,7 +1027,7 @@
         <v>5</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C4" s="17" t="s">
         <v>6</v>
@@ -1064,7 +1064,7 @@
         <v>10</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C7" s="17" t="s">
         <v>9</v>
@@ -1111,7 +1111,7 @@
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="str">
         <f>B3&amp;"-Web"</f>
-        <v>AXE_Test-Web</v>
+        <v>AXE_THAINGUYEN-Web</v>
       </c>
       <c r="B11" s="21" t="s">
         <v>17</v>
@@ -1122,7 +1122,7 @@
       <c r="G11" s="12"/>
       <c r="H11" s="21" t="str">
         <f>IF(A11="","",$B$8&amp;" add apppool /name:"&amp;A11&amp;" /managedRuntimeVersion:"&amp;B11&amp;" /managedPipelineMode:"&amp;C11&amp;"")</f>
-        <v>c:\Windows\system32\inetsrv\appcmd add apppool /name:AXE_Test-Web /managedRuntimeVersion:v4.0 /managedPipelineMode:Integrated</v>
+        <v>c:\Windows\system32\inetsrv\appcmd add apppool /name:AXE_THAINGUYEN-Web /managedRuntimeVersion:v4.0 /managedPipelineMode:Integrated</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
@@ -1169,27 +1169,27 @@
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="21" t="str">
         <f>B5&amp;"Web"</f>
-        <v>AXE_Test_Web</v>
+        <v>AXE_2026_THAINGUYEN_Web</v>
       </c>
       <c r="B15" s="21" t="str">
-        <f>$B$4&amp;"AXE-Dash"</f>
-        <v>E:\TestTool_Dựng web\AXE-Dash</v>
+        <f>$B$4&amp;"dard"</f>
+        <v>E:\Source_Web\AXE-2026-ThaiNguyen\dard</v>
       </c>
       <c r="C15" s="17" t="s">
         <v>25</v>
       </c>
       <c r="D15" s="16">
-        <v>1221</v>
+        <v>8539</v>
       </c>
       <c r="E15" s="21"/>
       <c r="F15" s="21" t="str">
         <f>A11</f>
-        <v>AXE_Test-Web</v>
+        <v>AXE_THAINGUYEN-Web</v>
       </c>
       <c r="G15" s="12"/>
       <c r="H15" s="21" t="str">
         <f>IF(A15="","",$B$8&amp;" add site /name:"""&amp;A15&amp;""" /physicalPath:"&amp;B15&amp;" /bindings:"&amp;C15&amp;"/*:"&amp;D15&amp;":"&amp;E15&amp;"" )</f>
-        <v>c:\Windows\system32\inetsrv\appcmd add site /name:"AXE_Test_Web" /physicalPath:E:\TestTool_Dựng web\AXE-Dash /bindings:http/*:1221:</v>
+        <v>c:\Windows\system32\inetsrv\appcmd add site /name:"AXE_2026_THAINGUYEN_Web" /physicalPath:E:\Source_Web\AXE-2026-ThaiNguyen\dard /bindings:http/*:8539:</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
@@ -1240,11 +1240,11 @@
       </c>
       <c r="B19" s="21" t="str">
         <f t="shared" ref="B19:B24" si="0">$A$15</f>
-        <v>AXE_Test_Web</v>
+        <v>AXE_2026_THAINGUYEN_Web</v>
       </c>
       <c r="C19" s="17" t="str">
-        <f>$B$4&amp;"AXE-Acc"</f>
-        <v>E:\TestTool_Dựng web\AXE-Acc</v>
+        <f>$B$4&amp;"login"</f>
+        <v>E:\Source_Web\AXE-2026-ThaiNguyen\login</v>
       </c>
       <c r="D19" s="22" t="s">
         <v>32</v>
@@ -1256,20 +1256,20 @@
       <c r="G19" s="12"/>
       <c r="H19" s="21" t="str">
         <f t="shared" ref="H19:H24" si="1">IF(D19="","",$B$8&amp;" add app  /site.name:"""&amp;B19&amp;""" /path:/"&amp;A19&amp;" /physicalPath:"&amp;C19&amp;"")</f>
-        <v>c:\Windows\system32\inetsrv\appcmd add app  /site.name:"AXE_Test_Web" /path:/login /physicalPath:E:\TestTool_Dựng web\AXE-Acc</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" ht="27.6" x14ac:dyDescent="0.25">
+        <v>c:\Windows\system32\inetsrv\appcmd add app  /site.name:"AXE_2026_THAINGUYEN_Web" /path:/login /physicalPath:E:\Source_Web\AXE-2026-ThaiNguyen\login</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="21" t="s">
         <v>34</v>
       </c>
       <c r="B20" s="21" t="str">
         <f t="shared" si="0"/>
-        <v>AXE_Test_Web</v>
+        <v>AXE_2026_THAINGUYEN_Web</v>
       </c>
       <c r="C20" s="17" t="str">
-        <f>$B$4&amp;"AXE-Admin"</f>
-        <v>E:\TestTool_Dựng web\AXE-Admin</v>
+        <f>$B$4&amp;"admin"</f>
+        <v>E:\Source_Web\AXE-2026-ThaiNguyen\admin</v>
       </c>
       <c r="D20" s="22" t="s">
         <v>32</v>
@@ -1281,20 +1281,20 @@
       <c r="G20" s="12"/>
       <c r="H20" s="21" t="str">
         <f t="shared" si="1"/>
-        <v>c:\Windows\system32\inetsrv\appcmd add app  /site.name:"AXE_Test_Web" /path:/admin /physicalPath:E:\TestTool_Dựng web\AXE-Admin</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" ht="27.6" x14ac:dyDescent="0.25">
+        <v>c:\Windows\system32\inetsrv\appcmd add app  /site.name:"AXE_2026_THAINGUYEN_Web" /path:/admin /physicalPath:E:\Source_Web\AXE-2026-ThaiNguyen\admin</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="21" t="s">
         <v>35</v>
       </c>
       <c r="B21" s="21" t="str">
         <f t="shared" si="0"/>
-        <v>AXE_Test_Web</v>
+        <v>AXE_2026_THAINGUYEN_Web</v>
       </c>
       <c r="C21" s="17" t="str">
-        <f>$B$4&amp;"AXE-ResumUploader"</f>
-        <v>E:\TestTool_Dựng web\AXE-ResumUploader</v>
+        <f>$B$4&amp;"resumable"</f>
+        <v>E:\Source_Web\AXE-2026-ThaiNguyen\resumable</v>
       </c>
       <c r="D21" s="22" t="s">
         <v>32</v>
@@ -1306,20 +1306,20 @@
       <c r="G21" s="12"/>
       <c r="H21" s="21" t="str">
         <f t="shared" si="1"/>
-        <v>c:\Windows\system32\inetsrv\appcmd add app  /site.name:"AXE_Test_Web" /path:/resumable /physicalPath:E:\TestTool_Dựng web\AXE-ResumUploader</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" ht="27.6" x14ac:dyDescent="0.25">
+        <v>c:\Windows\system32\inetsrv\appcmd add app  /site.name:"AXE_2026_THAINGUYEN_Web" /path:/resumable /physicalPath:E:\Source_Web\AXE-2026-ThaiNguyen\resumable</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="21" t="s">
         <v>36</v>
       </c>
       <c r="B22" s="21" t="str">
         <f t="shared" si="0"/>
-        <v>AXE_Test_Web</v>
+        <v>AXE_2026_THAINGUYEN_Web</v>
       </c>
       <c r="C22" s="17" t="str">
-        <f>$B$4&amp;"AXE-Uploader"</f>
-        <v>E:\TestTool_Dựng web\AXE-Uploader</v>
+        <f>$B$4&amp;"uploader"</f>
+        <v>E:\Source_Web\AXE-2026-ThaiNguyen\uploader</v>
       </c>
       <c r="D22" s="22" t="s">
         <v>32</v>
@@ -1331,20 +1331,20 @@
       <c r="G22" s="12"/>
       <c r="H22" s="21" t="str">
         <f t="shared" si="1"/>
-        <v>c:\Windows\system32\inetsrv\appcmd add app  /site.name:"AXE_Test_Web" /path:/uploader /physicalPath:E:\TestTool_Dựng web\AXE-Uploader</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+        <v>c:\Windows\system32\inetsrv\appcmd add app  /site.name:"AXE_2026_THAINGUYEN_Web" /path:/uploader /physicalPath:E:\Source_Web\AXE-2026-ThaiNguyen\uploader</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A23" s="21" t="s">
         <v>37</v>
       </c>
       <c r="B23" s="21" t="str">
         <f t="shared" si="0"/>
-        <v>AXE_Test_Web</v>
+        <v>AXE_2026_THAINGUYEN_Web</v>
       </c>
       <c r="C23" s="17" t="str">
         <f>$B$7</f>
-        <v>C:\Users\Admin\Desktop\Test</v>
+        <v>E:\DataStorage\StorageAXE-2026-ThaiNguyen\Storage</v>
       </c>
       <c r="D23" s="22" t="s">
         <v>32</v>
@@ -1356,20 +1356,20 @@
       <c r="G23" s="12"/>
       <c r="H23" s="21" t="str">
         <f t="shared" si="1"/>
-        <v>c:\Windows\system32\inetsrv\appcmd add app  /site.name:"AXE_Test_Web" /path:/storage /physicalPath:C:\Users\Admin\Desktop\Test</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" ht="27.6" x14ac:dyDescent="0.25">
+        <v>c:\Windows\system32\inetsrv\appcmd add app  /site.name:"AXE_2026_THAINGUYEN_Web" /path:/storage /physicalPath:E:\DataStorage\StorageAXE-2026-ThaiNguyen\Storage</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="21" t="s">
         <v>38</v>
       </c>
       <c r="B24" s="21" t="str">
         <f t="shared" si="0"/>
-        <v>AXE_Test_Web</v>
+        <v>AXE_2026_THAINGUYEN_Web</v>
       </c>
       <c r="C24" s="17" t="str">
-        <f>$B$4&amp;"AXE-SoHoa"</f>
-        <v>E:\TestTool_Dựng web\AXE-SoHoa</v>
+        <f>$B$4&amp;"sohoa"</f>
+        <v>E:\Source_Web\AXE-2026-ThaiNguyen\sohoa</v>
       </c>
       <c r="D24" s="16" t="s">
         <v>32</v>
@@ -1381,7 +1381,7 @@
       <c r="G24" s="12"/>
       <c r="H24" s="21" t="str">
         <f t="shared" si="1"/>
-        <v>c:\Windows\system32\inetsrv\appcmd add app  /site.name:"AXE_Test_Web" /path:/doc /physicalPath:E:\TestTool_Dựng web\AXE-SoHoa</v>
+        <v>c:\Windows\system32\inetsrv\appcmd add app  /site.name:"AXE_2026_THAINGUYEN_Web" /path:/doc /physicalPath:E:\Source_Web\AXE-2026-ThaiNguyen\sohoa</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
@@ -1420,16 +1420,16 @@
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="21" t="str">
         <f>$A$15</f>
-        <v>AXE_Test_Web</v>
+        <v>AXE_2026_THAINGUYEN_Web</v>
       </c>
       <c r="B28" s="21"/>
       <c r="C28" s="17" t="str">
         <f>$A$11</f>
-        <v>AXE_Test-Web</v>
+        <v>AXE_THAINGUYEN-Web</v>
       </c>
       <c r="H28" s="21" t="str">
         <f>IF(C28="","",$B$8&amp;" set app "&amp;A28&amp;"/  /"&amp;"applicationPool:"&amp;C28&amp;"")</f>
-        <v>c:\Windows\system32\inetsrv\appcmd set app AXE_Test_Web/  /applicationPool:AXE_Test-Web</v>
+        <v>c:\Windows\system32\inetsrv\appcmd set app AXE_2026_THAINGUYEN_Web/  /applicationPool:AXE_THAINGUYEN-Web</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
@@ -1469,121 +1469,121 @@
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="21" t="str">
         <f>$A$15</f>
-        <v>AXE_Test_Web</v>
+        <v>AXE_2026_THAINGUYEN_Web</v>
       </c>
       <c r="B32" s="21" t="s">
         <v>31</v>
       </c>
       <c r="C32" s="17" t="str">
         <f>$A$11</f>
-        <v>AXE_Test-Web</v>
+        <v>AXE_THAINGUYEN-Web</v>
       </c>
       <c r="D32" s="49"/>
       <c r="E32" s="49"/>
       <c r="F32" s="49"/>
       <c r="H32" s="21" t="str">
         <f>IF(C32="","",$B$8&amp;" set app "&amp;A32&amp;"/"&amp;B32&amp;"  /"&amp;"applicationPool:"&amp;C32&amp;"")</f>
-        <v>c:\Windows\system32\inetsrv\appcmd set app AXE_Test_Web/login  /applicationPool:AXE_Test-Web</v>
+        <v>c:\Windows\system32\inetsrv\appcmd set app AXE_2026_THAINGUYEN_Web/login  /applicationPool:AXE_THAINGUYEN-Web</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="21" t="str">
         <f t="shared" ref="A33:A37" si="2">$A$15</f>
-        <v>AXE_Test_Web</v>
+        <v>AXE_2026_THAINGUYEN_Web</v>
       </c>
       <c r="B33" s="21" t="s">
         <v>34</v>
       </c>
       <c r="C33" s="17" t="str">
         <f t="shared" ref="C33:C37" si="3">$A$11</f>
-        <v>AXE_Test-Web</v>
+        <v>AXE_THAINGUYEN-Web</v>
       </c>
       <c r="D33" s="43"/>
       <c r="E33" s="43"/>
       <c r="F33" s="43"/>
       <c r="H33" s="21" t="str">
         <f>IF(C33="","",$B$8&amp;" set app "&amp;A33&amp;"/"&amp;B33&amp;"  /"&amp;"applicationPool:"&amp;C33&amp;"")</f>
-        <v>c:\Windows\system32\inetsrv\appcmd set app AXE_Test_Web/admin  /applicationPool:AXE_Test-Web</v>
+        <v>c:\Windows\system32\inetsrv\appcmd set app AXE_2026_THAINGUYEN_Web/admin  /applicationPool:AXE_THAINGUYEN-Web</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>AXE_Test_Web</v>
+        <v>AXE_2026_THAINGUYEN_Web</v>
       </c>
       <c r="B34" s="21" t="s">
         <v>35</v>
       </c>
       <c r="C34" s="17" t="str">
         <f t="shared" si="3"/>
-        <v>AXE_Test-Web</v>
+        <v>AXE_THAINGUYEN-Web</v>
       </c>
       <c r="D34" s="43"/>
       <c r="E34" s="43"/>
       <c r="F34" s="43"/>
       <c r="H34" s="21" t="str">
         <f>IF(C34="","",$B$8&amp;" set app "&amp;A34&amp;"/"&amp;B34&amp;"  /"&amp;"applicationPool:"&amp;C34&amp;"")</f>
-        <v>c:\Windows\system32\inetsrv\appcmd set app AXE_Test_Web/resumable  /applicationPool:AXE_Test-Web</v>
+        <v>c:\Windows\system32\inetsrv\appcmd set app AXE_2026_THAINGUYEN_Web/resumable  /applicationPool:AXE_THAINGUYEN-Web</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>AXE_Test_Web</v>
+        <v>AXE_2026_THAINGUYEN_Web</v>
       </c>
       <c r="B35" s="21" t="s">
         <v>36</v>
       </c>
       <c r="C35" s="17" t="str">
         <f t="shared" si="3"/>
-        <v>AXE_Test-Web</v>
+        <v>AXE_THAINGUYEN-Web</v>
       </c>
       <c r="D35" s="43"/>
       <c r="E35" s="43"/>
       <c r="F35" s="43"/>
       <c r="H35" s="21" t="str">
         <f>IF(C35="","",$B$8&amp;" set app "&amp;A35&amp;"/"&amp;B35&amp;"  /"&amp;"applicationPool:"&amp;C35&amp;"")</f>
-        <v>c:\Windows\system32\inetsrv\appcmd set app AXE_Test_Web/uploader  /applicationPool:AXE_Test-Web</v>
+        <v>c:\Windows\system32\inetsrv\appcmd set app AXE_2026_THAINGUYEN_Web/uploader  /applicationPool:AXE_THAINGUYEN-Web</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>AXE_Test_Web</v>
+        <v>AXE_2026_THAINGUYEN_Web</v>
       </c>
       <c r="B36" s="21" t="s">
         <v>37</v>
       </c>
       <c r="C36" s="17" t="str">
         <f t="shared" si="3"/>
-        <v>AXE_Test-Web</v>
+        <v>AXE_THAINGUYEN-Web</v>
       </c>
       <c r="D36" s="43"/>
       <c r="E36" s="43"/>
       <c r="F36" s="43"/>
       <c r="H36" s="21" t="str">
         <f>IF(C36="","","c:\Windows\system32\inetsrv\appcmd set app "&amp;A36&amp;"/"&amp;B36&amp;"  /"&amp;"applicationPool:"&amp;C36&amp;"")</f>
-        <v>c:\Windows\system32\inetsrv\appcmd set app AXE_Test_Web/storage  /applicationPool:AXE_Test-Web</v>
+        <v>c:\Windows\system32\inetsrv\appcmd set app AXE_2026_THAINGUYEN_Web/storage  /applicationPool:AXE_THAINGUYEN-Web</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>AXE_Test_Web</v>
+        <v>AXE_2026_THAINGUYEN_Web</v>
       </c>
       <c r="B37" s="21" t="s">
         <v>38</v>
       </c>
       <c r="C37" s="17" t="str">
         <f t="shared" si="3"/>
-        <v>AXE_Test-Web</v>
+        <v>AXE_THAINGUYEN-Web</v>
       </c>
       <c r="D37" s="36"/>
       <c r="E37" s="37"/>
       <c r="F37" s="38"/>
       <c r="H37" s="21" t="str">
         <f t="shared" ref="H37:H38" si="4">IF(C37="","","c:\Windows\system32\inetsrv\appcmd set app "&amp;A37&amp;"/"&amp;B37&amp;"  /"&amp;"applicationPool:"&amp;C37&amp;"")</f>
-        <v>c:\Windows\system32\inetsrv\appcmd set app AXE_Test_Web/doc  /applicationPool:AXE_Test-Web</v>
+        <v>c:\Windows\system32\inetsrv\appcmd set app AXE_2026_THAINGUYEN_Web/doc  /applicationPool:AXE_THAINGUYEN-Web</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
@@ -2831,27 +2831,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Ghich_x00fa_ xmlns="97d068c0-5bfb-413b-9996-819e39fdf128" xsi:nil="true"/>
-    <TaxCatchAll xmlns="2c7f0914-2907-4374-a90b-da4fc7d9e6d0" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="97d068c0-5bfb-413b-9996-819e39fdf128">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010097FE9C0C8E574444875F1CBBF8414DDA" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c7e0992f45b677c2156c5ab52d17057f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="97d068c0-5bfb-413b-9996-819e39fdf128" xmlns:ns3="2c7f0914-2907-4374-a90b-da4fc7d9e6d0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2f06a3ea3329379ac3c4a4f5da7fed49" ns2:_="" ns3:_="">
     <xsd:import namespace="97d068c0-5bfb-413b-9996-819e39fdf128"/>
@@ -3086,26 +3065,28 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1FDEE16B-9D1D-4FD0-B127-E14D995BDF2D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EA8505A6-C0ED-439D-B023-AA9B1B1662BB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="97d068c0-5bfb-413b-9996-819e39fdf128"/>
-    <ds:schemaRef ds:uri="2c7f0914-2907-4374-a90b-da4fc7d9e6d0"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Ghich_x00fa_ xmlns="97d068c0-5bfb-413b-9996-819e39fdf128" xsi:nil="true"/>
+    <TaxCatchAll xmlns="2c7f0914-2907-4374-a90b-da4fc7d9e6d0" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="97d068c0-5bfb-413b-9996-819e39fdf128">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E3A15DF-6B1B-40AC-992D-CB264AF46DCF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3122,4 +3103,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1FDEE16B-9D1D-4FD0-B127-E14D995BDF2D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EA8505A6-C0ED-439D-B023-AA9B1B1662BB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="97d068c0-5bfb-413b-9996-819e39fdf128"/>
+    <ds:schemaRef ds:uri="2c7f0914-2907-4374-a90b-da4fc7d9e6d0"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>